<commit_message>
Update app.py and data files
</commit_message>
<xml_diff>
--- a/R sq.xlsx
+++ b/R sq.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\Desktop\TSD ML\TSD ML\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B31D0E8F-C135-45EE-9675-ECC5FD384803}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B440C370-F464-4F31-810D-724F5A79D7D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{60DAC5D0-9666-476F-B618-55591D7E2975}"/>
   </bookViews>
@@ -61,10 +61,17 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -78,7 +85,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -86,12 +93,29 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -406,77 +430,78 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E827957-05CD-448F-99DC-75BEDBE2B319}">
-  <dimension ref="A1:D5"/>
+  <dimension ref="B3:E7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13.90625" customWidth="1"/>
     <col min="2" max="2" width="12.90625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B1" t="s">
+    <row r="3" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B3" s="1"/>
+      <c r="C3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E3" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+    <row r="4" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B4" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B2">
+      <c r="C4" s="1">
         <v>0.84930000000000005</v>
       </c>
-      <c r="C2">
+      <c r="D4" s="1">
         <v>0.96209999999999996</v>
       </c>
-      <c r="D2">
+      <c r="E4" s="2">
         <v>0.99880000000000002</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
+    <row r="5" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B5" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B3">
+      <c r="C5" s="1">
         <v>47.833599999999997</v>
       </c>
-      <c r="C3">
+      <c r="D5" s="1">
         <v>12.0335</v>
       </c>
-      <c r="D3">
+      <c r="E5" s="2">
         <v>0.36649999999999999</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
+    <row r="6" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B6" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B4">
+      <c r="C6" s="1">
         <v>6.9161999999999999</v>
       </c>
-      <c r="C4">
+      <c r="D6" s="1">
         <v>3.4689000000000001</v>
       </c>
-      <c r="D4">
+      <c r="E6" s="2">
         <v>0.60540000000000005</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
+    <row r="7" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B7" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B5">
+      <c r="C7" s="1">
         <v>74.777500000000003</v>
       </c>
-      <c r="C5">
+      <c r="D7" s="1">
         <v>73.164599999999993</v>
       </c>
-      <c r="D5">
+      <c r="E7" s="2">
         <v>4.8963999999999999</v>
       </c>
     </row>

</xml_diff>